<commit_message>
Matrices con evidencia observada y comparacion con nivel de riesgo
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JwRbVrCmx8QHfMMhE96adb
</commit_message>
<xml_diff>
--- a/matrices/matriz_riesgos.xlsx
+++ b/matrices/matriz_riesgos.xlsx
@@ -238,7 +238,7 @@
     <t xml:space="preserve">Proteger (PR): PR.AA Gestión de identidades, autenticación y control de acceso. Detectar (DE): DE.CM Monitoreo continuo.</t>
   </si>
   <si>
-    <t xml:space="preserve">PENDIENTE: enlazar resultados de scripts/run_scenario.py (S1–S3) y extractos de auth.log (LOCKOUT_START/LOCKOUT_END).</t>
+    <t xml:space="preserve">OBSERVADO (22/10/2026): escenario S1–S3 en Apache y NGINX: sin controles 4.º fallo=401 y clave correcta durante la prueba=302; con controles 4.º fallo=429 y clave correcta durante el bloqueo=429, 302 al terminar. auth.log: LOCKOUT_START y LOCKOUT_END separados por 120 s. Ver evidence/resultados/, evidence/analisis/comparacion.md y capturas.</t>
   </si>
   <si>
     <t xml:space="preserve">Un ataque lento o distribuido (varias IP) puede quedar bajo el umbral; el bloqueo puede usarse para negar el servicio a la cuenta legítima. Acciones: límite por IP, MFA, alertas.</t>
@@ -253,7 +253,7 @@
     <t xml:space="preserve">Proteger (PR): PR.AT Concienciación y capacitación; PR.AA Autenticación. Detectar (DE): DE.AE Análisis de eventos adversos.</t>
   </si>
   <si>
-    <t xml:space="preserve">PENDIENTE: capturas del mensaje simulado, del enlace /r/qr1 y del evento LINK_VISIT en auth.log.</t>
+    <t xml:space="preserve">OBSERVADO: /r/qr1 redirige a /login?ref=afiche-qr y queda registrado LINK_VISIT con la campaña afiche-qr en auth.log (capturas del mensaje, QR, login y auth.log). NO observado: el efecto de MFA o capacitación (no implementados).</t>
   </si>
   <si>
     <t xml:space="preserve">Las credenciales capturadas siguen siendo válidas hasta el cambio; el bloqueo no impide el uso inmediato de una contraseña correcta. Acciones: MFA, capacitación periódica, filtrado de QR/enlaces.</t>
@@ -268,7 +268,7 @@
     <t xml:space="preserve">Detectar (DE): DE.CM Monitoreo continuo; DE.AE Análisis de eventos adversos.</t>
   </si>
   <si>
-    <t xml:space="preserve">PENDIENTE: extracto de auth.log y salida de scripts/analyze_logs.py que reconstruya la secuencia.</t>
+    <t xml:space="preserve">OBSERVADO: evidence/analisis/*_hardened.md reconstruye la secuencia y la correlación auditoría = access.log = ZAP = 7 intentos. Limitación observada: los intentos con usuario desconocido no cuentan para el bloqueo y el campo usuario se registra tal cual.</t>
   </si>
   <si>
     <t xml:space="preserve">Los registros están en el mismo host y sin protección de integridad. Acciones: envío a un servidor central/SIEM, retención y control de acceso a los logs.</t>
@@ -283,7 +283,7 @@
     <t xml:space="preserve">Proteger (PR): PR.PS Seguridad de la plataforma.</t>
   </si>
   <si>
-    <t xml:space="preserve">PENDIENTE: captura de los encabezados de respuesta antes/después (curl -I o ZAP).</t>
+    <t xml:space="preserve">OBSERVADO: curl -I a Apache muestra Server: Apache (sin gunicorn) y X-Content-Type-Options una sola vez. No se midió el estado «antes» con capturas.</t>
   </si>
   <si>
     <t xml:space="preserve">Siguen existiendo fallas desconocidas o de versión. Acciones: parches periódicos, TLS, escaneo de vulnerabilidades.</t>
@@ -292,7 +292,7 @@
     <t xml:space="preserve">Endurecimiento equivalente en NGINX: server_tokens off, proxy_hide_header Server, nosniff.</t>
   </si>
   <si>
-    <t xml:space="preserve">PENDIENTE: captura de los encabezados de respuesta antes/después.</t>
+    <t xml:space="preserve">OBSERVADO: curl -I a NGINX muestra Server: nginx (sin gunicorn) y X-Content-Type-Options una sola vez.</t>
   </si>
   <si>
     <t xml:space="preserve">Igual que R-04. Acciones: parches periódicos, TLS, escaneo de vulnerabilidades.</t>
@@ -307,7 +307,7 @@
     <t xml:space="preserve">Proteger (PR): PR.DS Seguridad de los datos (en tránsito).</t>
   </si>
   <si>
-    <t xml:space="preserve">PENDIENTE: captura de ZAP mostrando el POST /login en claro (campos enmascarados en el repositorio).</t>
+    <t xml:space="preserve">OBSERVADO: ZAP captura los POST http://…/login (HTTP sin cifrado); el CSV del repositorio enmascara los campos. Ningún control de cifrado implementado.</t>
   </si>
   <si>
     <t xml:space="preserve">El riesgo permanece igual: un control no implementado no reduce el riesgo. Acción: habilitar TLS en Apache y NGINX.</t>
@@ -1322,7 +1322,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
@@ -1368,7 +1368,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
         <v>20</v>
       </c>
@@ -1414,7 +1414,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
         <v>27</v>
       </c>
@@ -1460,7 +1460,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
         <v>34</v>
       </c>
@@ -1506,7 +1506,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
         <v>41</v>
       </c>
@@ -1552,7 +1552,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
         <v>46</v>
       </c>

</xml_diff>

<commit_message>
Matriz de riesgos actualizada y comparacion regenerada
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JwRbVrCmx8QHfMMhE96adb
</commit_message>
<xml_diff>
--- a/matrices/matriz_riesgos.xlsx
+++ b/matrices/matriz_riesgos.xlsx
@@ -26,12 +26,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="120">
-  <si>
-    <t xml:space="preserve">Matriz de riesgos INICIAL — Laboratorio de phishing y monitoreo (BORRADOR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valores de P e I = estimación inicial del equipo; justificarlos y ajustarlos con la evidencia. Nivel = Probabilidad × Impacto (escala 1–5). Umbrales en la hoja «Escala».</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="127">
+  <si>
+    <t xml:space="preserve">Matriz de riesgos INICIAL — Laboratorio de phishing y monitoreo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P e I son valoraciones del equipo (juicio profesional, no mediciones), cada una justificada: OBSERVADO = respaldado por evidencia del laboratorio; JUICIO = criterio del equipo sin medición. Nivel = Probabilidad × Impacto (escala 1–5). Umbrales en la hoja «Escala».</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -85,7 +85,7 @@
     <t xml:space="preserve">Contraseña almacenada con hash (PBKDF2) y mensaje de error genérico. Sin bloqueo ni registro de auditoría.</t>
   </si>
   <si>
-    <t xml:space="preserve">P=4: no hay límite de intentos y la herramienta de ataque es trivial. I=3: la cuenta es ficticia pero representa una cuenta de funcionario con acceso a servicios.</t>
+    <t xml:space="preserve">P=4 (OBSERVADO): en modo sin controles se ejecutaron 4 fallos seguidos y la clave correcta entró (302): no hay límite de intentos. I=3 (JUICIO): la cuenta es ficticia pero representa una cuenta de funcionario con acceso a servicios.</t>
   </si>
   <si>
     <t xml:space="preserve">R-02</t>
@@ -127,7 +127,7 @@
     <t xml:space="preserve">access.log del servidor web (IP, hora, método, código HTTP). Sin registro a nivel de aplicación.</t>
   </si>
   <si>
-    <t xml:space="preserve">P=4: sin auditoría el evento ocurre sin ser detectado. I=3: afecta la capacidad de respuesta y de rendir cuentas.</t>
+    <t xml:space="preserve">P=4 (OBSERVADO): en modo sin controles la app registró 0 eventos de autenticación; solo existía el access.log del servidor. I=3 (JUICIO): afecta la capacidad de respuesta y de rendir cuentas.</t>
   </si>
   <si>
     <t xml:space="preserve">R-04</t>
@@ -184,13 +184,13 @@
     <t xml:space="preserve">Red aislada del laboratorio (control de entorno, no de la aplicación).</t>
   </si>
   <si>
-    <t xml:space="preserve">P=3: requiere estar en la misma red. I=4: expone directamente las credenciales.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matriz de riesgos RESIDUAL — Laboratorio de phishing y monitoreo (BORRADOR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Misma escala y metodología que la matriz inicial. P e I se vuelven a estimar considerando la eficacia esperada de los controles; reemplazar «PENDIENTE» con la evidencia real del laboratorio. Un control no hace desaparecer el riesgo automáticamente.</t>
+    <t xml:space="preserve">P=3 (JUICIO): requiere estar en la misma red. I=4 (JUICIO): el tráfico es HTTP y ZAP lo captura en claro; expone directamente las credenciales.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matriz de riesgos RESIDUAL — Laboratorio de phishing y monitoreo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Misma escala y metodología que la matriz inicial. P e I residuales son valoraciones del equipo justificadas en la columna final (OBSERVADO = evidencia del laboratorio; JUICIO = criterio sin medición). Un control no hace desaparecer el riesgo automáticamente.</t>
   </si>
   <si>
     <t xml:space="preserve">Activo afectado</t>
@@ -229,6 +229,9 @@
     <t xml:space="preserve">Riesgo que permanece y acciones adicionales</t>
   </si>
   <si>
+    <t xml:space="preserve">Justificación de P e I residual (observado / juicio)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bloqueo temporal de la cuenta tras 3 intentos fallidos consecutivos (120 s) + mensaje informativo + registro de activación y fin del bloqueo.</t>
   </si>
   <si>
@@ -244,6 +247,9 @@
     <t xml:space="preserve">Un ataque lento o distribuido (varias IP) puede quedar bajo el umbral; el bloqueo puede usarse para negar el servicio a la cuenta legítima. Acciones: límite por IP, MFA, alertas.</t>
   </si>
   <si>
+    <t xml:space="preserve">P=3 (antes 4) — OBSERVADO: con controles solo caben 3 intentos por cada 120 s (≈90 por hora por cuenta) frente a intentos ilimitados sin controles (4.º fallo=401 y clave correcta=302). No baja a 2 porque un ataque lento sigue siendo posible y los usuarios desconocidos nunca se bloquean (auth.log, usuario «123»). I=3 sin cambio (JUICIO): el control no reduce el daño de una cuenta comprometida.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Control parcial en el laboratorio: registro del evento LINK_VISIT (campaña) y bloqueo de la cuenta; recomendado: MFA y capacitación con simulacros.</t>
   </si>
   <si>
@@ -259,6 +265,9 @@
     <t xml:space="preserve">Las credenciales capturadas siguen siendo válidas hasta el cambio; el bloqueo no impide el uso inmediato de una contraseña correcta. Acciones: MFA, capacitación periódica, filtrado de QR/enlaces.</t>
   </si>
   <si>
+    <t xml:space="preserve">P=3 (antes 4) — OBSERVADO: /r/qr1 sigue llevando al login y queda registrado (LINK_VISIT, afiche-qr), y el bloqueo limita adivinar; JUICIO: baja solo 1 punto porque no hay MFA ni filtrado y una clave entregada por el usuario sigue siendo válida. I=4 sin cambio.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Registro de auditoría de autenticación (JSON Lines) con fecha/hora, usuario ficticio, resultado, IP y estado de bloqueo, sin contraseñas ni tokens.</t>
   </si>
   <si>
@@ -274,6 +283,9 @@
     <t xml:space="preserve">Los registros están en el mismo host y sin protección de integridad. Acciones: envío a un servidor central/SIEM, retención y control de acceso a los logs.</t>
   </si>
   <si>
+    <t xml:space="preserve">P=3 (antes 4) — OBSERVADO: ahora la app registra 7 de 7 intentos (auditoría = access.log = ZAP). JUICIO: no baja más porque nadie revisa el log de forma automática ni hay alertas, y los registros están en el mismo host. I=3 sin cambio.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Endurecimiento de la configuración: ocultar la tecnología interna (encabezado Server), ServerTokens Prod, nosniff, TRACE deshabilitado.</t>
   </si>
   <si>
@@ -289,6 +301,9 @@
     <t xml:space="preserve">Siguen existiendo fallas desconocidas o de versión. Acciones: parches periódicos, TLS, escaneo de vulnerabilidades.</t>
   </si>
   <si>
+    <t xml:space="preserve">P=3 sin cambio — OBSERVADO: curl -I muestra Server: Apache sin gunicorn, es decir menos información de reconocimiento; pero no hay evidencia de que sea menos explotable, por eso no se baja. I=3 (JUICIO).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Endurecimiento equivalente en NGINX: server_tokens off, proxy_hide_header Server, nosniff.</t>
   </si>
   <si>
@@ -298,6 +313,9 @@
     <t xml:space="preserve">Igual que R-04. Acciones: parches periódicos, TLS, escaneo de vulnerabilidades.</t>
   </si>
   <si>
+    <t xml:space="preserve">P=3 sin cambio — OBSERVADO: curl -I muestra Server: nginx sin gunicorn; no hay evidencia de menor explotabilidad. I=3 (JUICIO).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ninguno implementado en el laboratorio (limitación). Recomendado: HTTPS con TLS y HSTS.</t>
   </si>
   <si>
@@ -311,6 +329,9 @@
   </si>
   <si>
     <t xml:space="preserve">El riesgo permanece igual: un control no implementado no reduce el riesgo. Acción: habilitar TLS en Apache y NGINX.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P=3 e I=4 sin cambio — OBSERVADO: ZAP captura los POST a http://…/login (sin cifrado); no se implementó ningún control. Un control no implementado no reduce el riesgo.</t>
   </si>
   <si>
     <t xml:space="preserve">Escala de valoración (definida en la práctica)</t>
@@ -1003,7 +1024,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
@@ -1255,7 +1276,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -1269,6 +1290,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1321,6 +1343,9 @@
       <c r="M4" s="3" t="s">
         <v>66</v>
       </c>
+      <c r="N4" s="3" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
@@ -1331,26 +1356,26 @@
         <v>Cuenta de usuario ficticia «usuario.demo» en la aplicación de autenticación (formulario /login)</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H5" s="6" t="n">
         <v>3</v>
       </c>
       <c r="I5" s="6" t="n">
         <f aca="false">G5*H5</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J5" s="6" t="str">
         <f aca="false">LOOKUP(I5,Escala!$A$12:$A$15,Escala!$B$12:$B$15)</f>
@@ -1362,10 +1387,13 @@
       </c>
       <c r="L5" s="6" t="n">
         <f aca="false">I5-K5</f>
-        <v>-6</v>
+        <v>-3</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1377,16 +1405,16 @@
         <v>Cuenta de usuario ficticia (credenciales del funcionario) expuesta a un mensaje con QR / enlace corto</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G6" s="6" t="n">
         <v>3</v>
@@ -1411,7 +1439,10 @@
         <v>-4</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1423,26 +1454,26 @@
         <v>Registros de acceso: auth.log de la aplicación y access.log de Apache/NGINX</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H7" s="6" t="n">
         <v>3</v>
       </c>
       <c r="I7" s="6" t="n">
         <f aca="false">G7*H7</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J7" s="6" t="str">
         <f aca="false">LOOKUP(I7,Escala!$A$12:$A$15,Escala!$B$12:$B$15)</f>
@@ -1454,10 +1485,13 @@
       </c>
       <c r="L7" s="6" t="n">
         <f aca="false">I7-K7</f>
-        <v>-6</v>
+        <v>-3</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>81</v>
+        <v>84</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1469,26 +1503,26 @@
         <v>Servidor web Apache HTTP Server (proxy inverso de la aplicación)</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H8" s="6" t="n">
         <v>3</v>
       </c>
       <c r="I8" s="6" t="n">
         <f aca="false">G8*H8</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J8" s="6" t="str">
         <f aca="false">LOOKUP(I8,Escala!$A$12:$A$15,Escala!$B$12:$B$15)</f>
@@ -1500,10 +1534,13 @@
       </c>
       <c r="L8" s="6" t="n">
         <f aca="false">I8-K8</f>
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>86</v>
+        <v>90</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1515,26 +1552,26 @@
         <v>Servidor web NGINX (proxy inverso de la aplicación)</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>83</v>
-      </c>
       <c r="E9" s="5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
         <f aca="false">G9*H9</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J9" s="6" t="str">
         <f aca="false">LOOKUP(I9,Escala!$A$12:$A$15,Escala!$B$12:$B$15)</f>
@@ -1546,10 +1583,13 @@
       </c>
       <c r="L9" s="6" t="n">
         <f aca="false">I9-K9</f>
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>89</v>
+        <v>94</v>
+      </c>
+      <c r="N9" s="5" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1561,16 +1601,16 @@
         <v>Tráfico HTTP de autenticación (credenciales en tránsito entre cliente y servidor)</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="G10" s="6" t="n">
         <v>3</v>
@@ -1595,7 +1635,10 @@
         <v>0</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>94</v>
+        <v>100</v>
+      </c>
+      <c r="N10" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1637,18 +1680,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1656,10 +1699,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1667,10 +1710,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1678,10 +1721,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1689,10 +1732,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1700,26 +1743,26 @@
         <v>5</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1727,10 +1770,10 @@
         <v>1</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1738,10 +1781,10 @@
         <v>5</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1749,10 +1792,10 @@
         <v>10</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1760,15 +1803,15 @@
         <v>17</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>